<commit_message>
Add full  year profile and storage to enet.
</commit_message>
<xml_diff>
--- a/power-systems-ops/data/encoord/enet39.xlsx
+++ b/power-systems-ops/data/encoord/enet39.xlsx
@@ -12,20 +12,23 @@
     <sheet sheetId="8" name="LI" state="visible" r:id="rId8"/>
     <sheet sheetId="9" name="TRF" state="visible" r:id="rId9"/>
     <sheet sheetId="10" name="EDEM" state="visible" r:id="rId10"/>
-    <sheet sheetId="11" name="SHT" state="visible" r:id="rId11"/>
-    <sheet sheetId="12" name="WIND" state="visible" r:id="rId12"/>
-    <sheet sheetId="13" name="PV" state="visible" r:id="rId13"/>
-    <sheet sheetId="14" name="FUEL" state="visible" r:id="rId14"/>
-    <sheet sheetId="15" name="FGEN" state="visible" r:id="rId15"/>
-    <sheet sheetId="16" name="ASVC" state="visible" r:id="rId16"/>
-    <sheet sheetId="17" name="ASVCX" state="visible" r:id="rId17"/>
-    <sheet sheetId="18" name="EGRPM" state="visible" r:id="rId18"/>
+    <sheet sheetId="11" name="ESTR" state="visible" r:id="rId11"/>
+    <sheet sheetId="12" name="SHT" state="visible" r:id="rId12"/>
+    <sheet sheetId="13" name="WIND" state="visible" r:id="rId13"/>
+    <sheet sheetId="14" name="PV" state="visible" r:id="rId14"/>
+    <sheet sheetId="15" name="FUEL" state="visible" r:id="rId15"/>
+    <sheet sheetId="16" name="FGEN" state="visible" r:id="rId16"/>
+    <sheet sheetId="17" name="ASVC" state="visible" r:id="rId17"/>
+    <sheet sheetId="18" name="ASVCX" state="visible" r:id="rId18"/>
+    <sheet sheetId="19" name="ECNSTR" state="visible" r:id="rId19"/>
+    <sheet sheetId="20" name="EVAR" state="visible" r:id="rId20"/>
+    <sheet sheetId="21" name="EGRPM" state="visible" r:id="rId21"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1652">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1702">
   <si>
     <t>Extension</t>
   </si>
@@ -4656,6 +4659,90 @@
     <t>QMINDEF [MVAr] = -∞</t>
   </si>
   <si>
+    <t>ESTR_0</t>
+  </si>
+  <si>
+    <t>GENPHASES  = ABC</t>
+  </si>
+  <si>
+    <t>MaxCapDef [MJ] = ∞</t>
+  </si>
+  <si>
+    <t>MaxDownRampDef [MW/min] = ∞</t>
+  </si>
+  <si>
+    <t>MaxUpRampDef [MW/min] = ∞</t>
+  </si>
+  <si>
+    <t>MinDownTimeDDDef [h] = 0</t>
+  </si>
+  <si>
+    <t>MinDownTimeDGDef [h] = 0</t>
+  </si>
+  <si>
+    <t>MinDownTimeGDDef [h] = 0</t>
+  </si>
+  <si>
+    <t>MinDownTimeGGDef [h] = 0</t>
+  </si>
+  <si>
+    <t>MinUpTimeDDef [h] = 0</t>
+  </si>
+  <si>
+    <t>MinUpTimeGDef [h] = 0</t>
+  </si>
+  <si>
+    <t>PDeff [-] = 1</t>
+  </si>
+  <si>
+    <t>PDMAXDEF [MW] = ∞</t>
+  </si>
+  <si>
+    <t>PDMAXPRCDEF [$/MWh] = ∞</t>
+  </si>
+  <si>
+    <t>PDMINDEF [MW] = 0</t>
+  </si>
+  <si>
+    <t>PDMINPRCDEF [$/MWh] = ∞</t>
+  </si>
+  <si>
+    <t>PFSETDEF [-] = 0</t>
+  </si>
+  <si>
+    <t>PGeff [-] = 1</t>
+  </si>
+  <si>
+    <t>PGMAXDEF [MW] = ∞</t>
+  </si>
+  <si>
+    <t>PGMAXPRCDEF [$/MWh] = ∞</t>
+  </si>
+  <si>
+    <t>PGMINDEF [MW] = 0</t>
+  </si>
+  <si>
+    <t>PGMINPRCDEF [$/MWh] = ∞</t>
+  </si>
+  <si>
+    <t>QSETDEF [MVAr] = 0</t>
+  </si>
+  <si>
+    <t>SOCMAXPRCDEF [$/MWh] = 1000000</t>
+  </si>
+  <si>
+    <t>SOCMINPRCDEF [$/MWh] = 1000000</t>
+  </si>
+  <si>
+    <t>SOCSETPRCDEF [$/MWh] = 1000000</t>
+  </si>
+  <si>
+    <t>VOMDPriceDef [$/MWh] = 0</t>
+  </si>
+  <si>
+    <t>VOMGPriceDef [$/MWh] = 0</t>
+  </si>
+  <si>
     <t>SHUNT_0</t>
   </si>
   <si>
@@ -4704,18 +4791,6 @@
     <t>LOSSES [%] = 14.08</t>
   </si>
   <si>
-    <t>MaxDownRampDef [MW/min] = ∞</t>
-  </si>
-  <si>
-    <t>MaxUpRampDef [MW/min] = ∞</t>
-  </si>
-  <si>
-    <t>PFSETDEF [-] = 0</t>
-  </si>
-  <si>
-    <t>QSETDEF [MVAr] = 0</t>
-  </si>
-  <si>
     <t>RRN [pu] = 0</t>
   </si>
   <si>
@@ -4758,9 +4833,6 @@
     <t>DCACRatio [-] = 1.1</t>
   </si>
   <si>
-    <t>GENPHASES  = ABC</t>
-  </si>
-  <si>
     <t>IMAXPU [pu] = 1.1</t>
   </si>
   <si>
@@ -4779,6 +4851,24 @@
     <t>VMINPU [pu] = 0.9</t>
   </si>
   <si>
+    <t>WeatherData\Solar_ad4505ee460147bc8e869230fe60b076_41.76312_-72.78442_2021_60.P3Sr.csv</t>
+  </si>
+  <si>
+    <t>WeatherData\Solar_2b2bc61028964557870e8f9cd92cc5d3_41.47978_-73.19092_2021_60.P3Sr.csv</t>
+  </si>
+  <si>
+    <t>WeatherData\Solar_a2069d4a8c67454394c42c4db24ab6c0_41.69753_-71.14197_2021_60.P3Sr.csv</t>
+  </si>
+  <si>
+    <t>WeatherData\Solar_a30c0835544f41bf92e1a0dade6d81da_42.25495_-70.98816_2021_60.P3Sr.csv</t>
+  </si>
+  <si>
+    <t>WeatherData\Solar_b1ec062780e04f15b9089ffb2c7a9340_42.5126_-71.53473_2021_60.P3Sr.csv</t>
+  </si>
+  <si>
+    <t>WeatherData\Solar_d0b3e295c8b74c5fa3ecbf1957b375fd_44.09548_-69.85107_2021_60.P3Sr.csv</t>
+  </si>
+  <si>
     <t>URANIUM</t>
   </si>
   <si>
@@ -4948,6 +5038,69 @@
   </si>
   <si>
     <t>FGEN.DANSKAMMER</t>
+  </si>
+  <si>
+    <t>ECNSTR_0</t>
+  </si>
+  <si>
+    <t>ECNSTR_1</t>
+  </si>
+  <si>
+    <t>ECNSTR_2</t>
+  </si>
+  <si>
+    <t>ECNSTR_3</t>
+  </si>
+  <si>
+    <t>ECNSTR_4</t>
+  </si>
+  <si>
+    <t>AvgLowBoundDef [-] = -∞</t>
+  </si>
+  <si>
+    <t>AvgUpBoundDef [-] = ∞</t>
+  </si>
+  <si>
+    <t>LowBoundDef [-] = -∞</t>
+  </si>
+  <si>
+    <t>UpBoundDef [-] = ∞</t>
+  </si>
+  <si>
+    <t>EVAR_0</t>
+  </si>
+  <si>
+    <t>EVAR_1</t>
+  </si>
+  <si>
+    <t>EVAR_2</t>
+  </si>
+  <si>
+    <t>EVAR_3</t>
+  </si>
+  <si>
+    <t>EVAR_4</t>
+  </si>
+  <si>
+    <t>CoeffDef [-] = 1</t>
+  </si>
+  <si>
+    <t>InService  = False</t>
+  </si>
+  <si>
+    <t>ObjVarName  = NONE</t>
+  </si>
+  <si>
+    <t>PG</t>
+  </si>
+  <si>
+    <t>PD</t>
+  </si>
+  <si>
+    <t>SOC</t>
+  </si>
+  <si>
+    <t>ESTR.ESTR_0</t>
   </si>
   <si>
     <t>FGEN.MILLSTONE</t>
@@ -17476,6 +17629,280 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:AK2"/>
+  <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" width="6.93359375" hidden="false" outlineLevel="0"/>
+    <col min="2" max="2" bestFit="true" width="15.19140625" hidden="false" outlineLevel="0"/>
+    <col min="3" max="3" bestFit="true" width="4.7109375" hidden="false" outlineLevel="0"/>
+    <col min="4" max="4" bestFit="true" width="16.87109375" hidden="false" outlineLevel="0"/>
+    <col min="5" max="5" bestFit="true" width="4.03125" hidden="false" outlineLevel="0"/>
+    <col min="6" max="6" bestFit="true" width="14.68359375" hidden="false" outlineLevel="0"/>
+    <col min="7" max="7" bestFit="true" width="18.5625" hidden="false" outlineLevel="0"/>
+    <col min="8" max="8" bestFit="true" width="30.50390625" hidden="false" outlineLevel="0"/>
+    <col min="9" max="9" bestFit="true" width="27.9609375" hidden="false" outlineLevel="0"/>
+    <col min="10" max="10" bestFit="true" width="24.73046875" hidden="false" outlineLevel="0"/>
+    <col min="11" max="12" bestFit="true" width="24.76171875" hidden="false" outlineLevel="0"/>
+    <col min="13" max="13" bestFit="true" width="24.79296875" hidden="false" outlineLevel="0"/>
+    <col min="14" max="14" bestFit="true" width="20.90234375" hidden="false" outlineLevel="0"/>
+    <col min="15" max="15" bestFit="true" width="20.93359375" hidden="false" outlineLevel="0"/>
+    <col min="16" max="16" bestFit="true" width="10.78125" hidden="false" outlineLevel="0"/>
+    <col min="17" max="17" bestFit="true" width="19.640625" hidden="false" outlineLevel="0"/>
+    <col min="18" max="18" bestFit="true" width="25.93359375" hidden="false" outlineLevel="0"/>
+    <col min="19" max="19" bestFit="true" width="18.4921875" hidden="false" outlineLevel="0"/>
+    <col min="20" max="20" bestFit="true" width="25.51171875" hidden="false" outlineLevel="0"/>
+    <col min="21" max="21" bestFit="true" width="14.4609375" hidden="false" outlineLevel="0"/>
+    <col min="22" max="22" bestFit="true" width="10.8125" hidden="false" outlineLevel="0"/>
+    <col min="23" max="23" bestFit="true" width="19.671875" hidden="false" outlineLevel="0"/>
+    <col min="24" max="24" bestFit="true" width="25.9609375" hidden="false" outlineLevel="0"/>
+    <col min="25" max="25" bestFit="true" width="18.53125" hidden="false" outlineLevel="0"/>
+    <col min="26" max="26" bestFit="true" width="25.54296875" hidden="false" outlineLevel="0"/>
+    <col min="27" max="27" bestFit="true" width="16.54296875" hidden="false" outlineLevel="0"/>
+    <col min="28" max="28" bestFit="true" width="26.0234375" hidden="false" outlineLevel="0"/>
+    <col min="29" max="29" bestFit="true" width="19.8515625" hidden="false" outlineLevel="0"/>
+    <col min="30" max="30" bestFit="true" width="20.07421875" hidden="false" outlineLevel="0"/>
+    <col min="31" max="31" bestFit="true" width="18.04296875" hidden="false" outlineLevel="0"/>
+    <col min="32" max="32" bestFit="true" width="32.671875" hidden="false" outlineLevel="0"/>
+    <col min="33" max="33" bestFit="true" width="32.25390625" hidden="false" outlineLevel="0"/>
+    <col min="34" max="34" bestFit="true" width="31.59375" hidden="false" outlineLevel="0"/>
+    <col min="35" max="35" bestFit="true" width="12.53125" hidden="false" outlineLevel="0"/>
+    <col min="36" max="36" bestFit="true" width="24.953125" hidden="false" outlineLevel="0"/>
+    <col min="37" max="37" bestFit="true" width="24.9921875" hidden="false" outlineLevel="0"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1544</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1414</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1545</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1546</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1547</v>
+      </c>
+      <c r="J1" t="s">
+        <v>1548</v>
+      </c>
+      <c r="K1" t="s">
+        <v>1549</v>
+      </c>
+      <c r="L1" t="s">
+        <v>1550</v>
+      </c>
+      <c r="M1" t="s">
+        <v>1551</v>
+      </c>
+      <c r="N1" t="s">
+        <v>1552</v>
+      </c>
+      <c r="O1" t="s">
+        <v>1553</v>
+      </c>
+      <c r="P1" t="s">
+        <v>1554</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>1555</v>
+      </c>
+      <c r="R1" t="s">
+        <v>1556</v>
+      </c>
+      <c r="S1" t="s">
+        <v>1557</v>
+      </c>
+      <c r="T1" t="s">
+        <v>1558</v>
+      </c>
+      <c r="U1" t="s">
+        <v>1559</v>
+      </c>
+      <c r="V1" t="s">
+        <v>1560</v>
+      </c>
+      <c r="W1" t="s">
+        <v>1561</v>
+      </c>
+      <c r="X1" t="s">
+        <v>1562</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>1563</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>1564</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>1536</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>1537</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>1541</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>1542</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>1565</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>1566</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>1567</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>1568</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>1415</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>1569</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>1570</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>1543</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1324</v>
+      </c>
+      <c r="D2" t="s">
+        <v>735</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1324</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>796</v>
+      </c>
+      <c r="H2" t="s">
+        <v>796</v>
+      </c>
+      <c r="I2" t="s">
+        <v>796</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>796</v>
+      </c>
+      <c r="R2" t="s">
+        <v>796</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="s">
+        <v>796</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="W2" t="s">
+        <v>796</v>
+      </c>
+      <c r="X2" t="s">
+        <v>796</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>796</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>796</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>795</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="AI2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:J3"/>
   <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
   <cols>
@@ -17502,10 +17929,10 @@
         <v>11</v>
       </c>
       <c r="D1" t="s">
-        <v>1545</v>
+        <v>1573</v>
       </c>
       <c r="E1" t="s">
-        <v>1546</v>
+        <v>1574</v>
       </c>
       <c r="F1" t="s">
         <v>6</v>
@@ -17517,7 +17944,7 @@
         <v>1471</v>
       </c>
       <c r="I1" t="s">
-        <v>1547</v>
+        <v>1575</v>
       </c>
       <c r="J1" t="s">
         <v>1415</v>
@@ -17525,7 +17952,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1543</v>
+        <v>1571</v>
       </c>
       <c r="B2" t="s">
         <v>1337</v>
@@ -17557,7 +17984,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1544</v>
+        <v>1572</v>
       </c>
       <c r="B3" t="s">
         <v>1338</v>
@@ -17592,7 +18019,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:AI4"/>
   <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
@@ -17645,19 +18072,19 @@
         <v>11</v>
       </c>
       <c r="D1" t="s">
-        <v>1551</v>
+        <v>1579</v>
       </c>
       <c r="E1" t="s">
-        <v>1552</v>
+        <v>1580</v>
       </c>
       <c r="F1" t="s">
-        <v>1553</v>
+        <v>1581</v>
       </c>
       <c r="G1" t="s">
-        <v>1554</v>
+        <v>1582</v>
       </c>
       <c r="H1" t="s">
-        <v>1555</v>
+        <v>1583</v>
       </c>
       <c r="I1" t="s">
         <v>6</v>
@@ -17666,22 +18093,22 @@
         <v>1414</v>
       </c>
       <c r="K1" t="s">
-        <v>1556</v>
+        <v>1584</v>
       </c>
       <c r="L1" t="s">
-        <v>1557</v>
+        <v>1585</v>
       </c>
       <c r="M1" t="s">
-        <v>1558</v>
+        <v>1586</v>
       </c>
       <c r="N1" t="s">
+        <v>1546</v>
+      </c>
+      <c r="O1" t="s">
+        <v>1547</v>
+      </c>
+      <c r="P1" t="s">
         <v>1559</v>
-      </c>
-      <c r="O1" t="s">
-        <v>1560</v>
-      </c>
-      <c r="P1" t="s">
-        <v>1561</v>
       </c>
       <c r="Q1" t="s">
         <v>1465</v>
@@ -17708,7 +18135,7 @@
         <v>1542</v>
       </c>
       <c r="Y1" t="s">
-        <v>1562</v>
+        <v>1565</v>
       </c>
       <c r="Z1" t="s">
         <v>1469</v>
@@ -17717,16 +18144,16 @@
         <v>1471</v>
       </c>
       <c r="AB1" t="s">
-        <v>1563</v>
+        <v>1587</v>
       </c>
       <c r="AC1" t="s">
-        <v>1564</v>
+        <v>1588</v>
       </c>
       <c r="AD1" t="s">
         <v>1415</v>
       </c>
       <c r="AE1" t="s">
-        <v>1565</v>
+        <v>1589</v>
       </c>
       <c r="AF1" t="s">
         <v>128</v>
@@ -17735,15 +18162,15 @@
         <v>129</v>
       </c>
       <c r="AH1" t="s">
-        <v>1566</v>
+        <v>1590</v>
       </c>
       <c r="AI1" t="s">
-        <v>1567</v>
+        <v>1591</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1548</v>
+        <v>1576</v>
       </c>
       <c r="B2" t="s">
         <v>1352</v>
@@ -17850,7 +18277,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1549</v>
+        <v>1577</v>
       </c>
       <c r="B3" t="s">
         <v>1355</v>
@@ -17957,7 +18384,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1550</v>
+        <v>1578</v>
       </c>
       <c r="B4" t="s">
         <v>1362</v>
@@ -18067,7 +18494,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:AM7"/>
   <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
@@ -18109,7 +18536,7 @@
     <col min="36" max="36" bestFit="true" width="17.0234375" hidden="false" outlineLevel="0"/>
     <col min="37" max="37" bestFit="true" width="16.6015625" hidden="false" outlineLevel="0"/>
     <col min="38" max="38" bestFit="true" width="23.6640625" hidden="false" outlineLevel="0"/>
-    <col min="39" max="39" bestFit="true" width="6.83203125" hidden="false" outlineLevel="0"/>
+    <col min="39" max="39" bestFit="true" width="85.921875" hidden="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18123,31 +18550,31 @@
         <v>11</v>
       </c>
       <c r="D1" t="s">
-        <v>1574</v>
+        <v>1598</v>
       </c>
       <c r="E1" t="s">
-        <v>1575</v>
+        <v>1599</v>
       </c>
       <c r="F1" t="s">
-        <v>1551</v>
+        <v>1579</v>
       </c>
       <c r="G1" t="s">
-        <v>1552</v>
+        <v>1580</v>
       </c>
       <c r="H1" t="s">
-        <v>1553</v>
+        <v>1581</v>
       </c>
       <c r="I1" t="s">
-        <v>1554</v>
+        <v>1582</v>
       </c>
       <c r="J1" t="s">
-        <v>1576</v>
+        <v>1600</v>
       </c>
       <c r="K1" t="s">
-        <v>1577</v>
+        <v>1544</v>
       </c>
       <c r="L1" t="s">
-        <v>1578</v>
+        <v>1601</v>
       </c>
       <c r="M1" t="s">
         <v>6</v>
@@ -18156,28 +18583,28 @@
         <v>1414</v>
       </c>
       <c r="O1" t="s">
-        <v>1579</v>
+        <v>1602</v>
       </c>
       <c r="P1" t="s">
-        <v>1556</v>
+        <v>1584</v>
       </c>
       <c r="Q1" t="s">
-        <v>1557</v>
+        <v>1585</v>
       </c>
       <c r="R1" t="s">
-        <v>1558</v>
+        <v>1586</v>
       </c>
       <c r="S1" t="s">
+        <v>1546</v>
+      </c>
+      <c r="T1" t="s">
+        <v>1547</v>
+      </c>
+      <c r="U1" t="s">
+        <v>1603</v>
+      </c>
+      <c r="V1" t="s">
         <v>1559</v>
-      </c>
-      <c r="T1" t="s">
-        <v>1560</v>
-      </c>
-      <c r="U1" t="s">
-        <v>1580</v>
-      </c>
-      <c r="V1" t="s">
-        <v>1561</v>
       </c>
       <c r="W1" t="s">
         <v>1465</v>
@@ -18204,7 +18631,7 @@
         <v>1542</v>
       </c>
       <c r="AE1" t="s">
-        <v>1562</v>
+        <v>1565</v>
       </c>
       <c r="AF1" t="s">
         <v>1469</v>
@@ -18213,19 +18640,19 @@
         <v>1471</v>
       </c>
       <c r="AH1" t="s">
-        <v>1581</v>
+        <v>1604</v>
       </c>
       <c r="AI1" t="s">
         <v>1415</v>
       </c>
       <c r="AJ1" t="s">
-        <v>1582</v>
+        <v>1605</v>
       </c>
       <c r="AK1" t="s">
-        <v>1583</v>
+        <v>1606</v>
       </c>
       <c r="AL1" t="s">
-        <v>1565</v>
+        <v>1589</v>
       </c>
       <c r="AM1" t="s">
         <v>128</v>
@@ -18233,7 +18660,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1568</v>
+        <v>1592</v>
       </c>
       <c r="B2" t="s">
         <v>1337</v>
@@ -18347,12 +18774,12 @@
         <v>0</v>
       </c>
       <c r="AM2" t="s">
-        <v>1324</v>
+        <v>1607</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1569</v>
+        <v>1593</v>
       </c>
       <c r="B3" t="s">
         <v>1341</v>
@@ -18466,12 +18893,12 @@
         <v>0</v>
       </c>
       <c r="AM3" t="s">
-        <v>1324</v>
+        <v>1608</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1570</v>
+        <v>1594</v>
       </c>
       <c r="B4" t="s">
         <v>1353</v>
@@ -18585,12 +19012,12 @@
         <v>0</v>
       </c>
       <c r="AM4" t="s">
-        <v>1324</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1571</v>
+        <v>1595</v>
       </c>
       <c r="B5" t="s">
         <v>1357</v>
@@ -18704,12 +19131,12 @@
         <v>0</v>
       </c>
       <c r="AM5" t="s">
-        <v>1324</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1572</v>
+        <v>1596</v>
       </c>
       <c r="B6" t="s">
         <v>1360</v>
@@ -18823,12 +19250,12 @@
         <v>0</v>
       </c>
       <c r="AM6" t="s">
-        <v>1324</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>1573</v>
+        <v>1597</v>
       </c>
       <c r="B7" t="s">
         <v>1362</v>
@@ -18942,7 +19369,7 @@
         <v>0</v>
       </c>
       <c r="AM7" t="s">
-        <v>1324</v>
+        <v>1612</v>
       </c>
     </row>
   </sheetData>
@@ -18950,7 +19377,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:I4"/>
   <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
@@ -18974,13 +19401,13 @@
         <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>1586</v>
+        <v>1615</v>
       </c>
       <c r="D1" t="s">
-        <v>1587</v>
+        <v>1616</v>
       </c>
       <c r="E1" t="s">
-        <v>1588</v>
+        <v>1617</v>
       </c>
       <c r="F1" t="s">
         <v>6</v>
@@ -18989,15 +19416,15 @@
         <v>1414</v>
       </c>
       <c r="H1" t="s">
-        <v>1589</v>
+        <v>1618</v>
       </c>
       <c r="I1" t="s">
-        <v>1590</v>
+        <v>1619</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1584</v>
+        <v>1613</v>
       </c>
       <c r="B2" t="s">
         <v>1324</v>
@@ -19026,7 +19453,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1585</v>
+        <v>1614</v>
       </c>
       <c r="B3" t="s">
         <v>1324</v>
@@ -19087,7 +19514,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:AR11"/>
   <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
@@ -19152,43 +19579,43 @@
         <v>11</v>
       </c>
       <c r="E1" t="s">
-        <v>1551</v>
+        <v>1579</v>
       </c>
       <c r="F1" t="s">
-        <v>1552</v>
+        <v>1580</v>
       </c>
       <c r="G1" t="s">
-        <v>1553</v>
+        <v>1581</v>
       </c>
       <c r="H1" t="s">
-        <v>1554</v>
+        <v>1582</v>
       </c>
       <c r="I1" t="s">
-        <v>1601</v>
+        <v>1630</v>
       </c>
       <c r="J1" t="s">
-        <v>1602</v>
+        <v>1631</v>
       </c>
       <c r="K1" t="s">
-        <v>1603</v>
+        <v>1632</v>
       </c>
       <c r="L1" t="s">
-        <v>1604</v>
+        <v>1633</v>
       </c>
       <c r="M1" t="s">
-        <v>1605</v>
+        <v>1634</v>
       </c>
       <c r="N1" t="s">
-        <v>1606</v>
+        <v>1635</v>
       </c>
       <c r="O1" t="s">
-        <v>1608</v>
+        <v>1637</v>
       </c>
       <c r="P1" t="s">
-        <v>1609</v>
+        <v>1638</v>
       </c>
       <c r="Q1" t="s">
-        <v>1610</v>
+        <v>1639</v>
       </c>
       <c r="R1" t="s">
         <v>6</v>
@@ -19197,22 +19624,22 @@
         <v>1414</v>
       </c>
       <c r="T1" t="s">
+        <v>1546</v>
+      </c>
+      <c r="U1" t="s">
+        <v>1547</v>
+      </c>
+      <c r="V1" t="s">
+        <v>1640</v>
+      </c>
+      <c r="W1" t="s">
+        <v>1641</v>
+      </c>
+      <c r="X1" t="s">
+        <v>1642</v>
+      </c>
+      <c r="Y1" t="s">
         <v>1559</v>
-      </c>
-      <c r="U1" t="s">
-        <v>1560</v>
-      </c>
-      <c r="V1" t="s">
-        <v>1611</v>
-      </c>
-      <c r="W1" t="s">
-        <v>1612</v>
-      </c>
-      <c r="X1" t="s">
-        <v>1613</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>1561</v>
       </c>
       <c r="Z1" t="s">
         <v>1465</v>
@@ -19245,16 +19672,16 @@
         <v>1471</v>
       </c>
       <c r="AJ1" t="s">
-        <v>1563</v>
+        <v>1587</v>
       </c>
       <c r="AK1" t="s">
-        <v>1564</v>
+        <v>1588</v>
       </c>
       <c r="AL1" t="s">
-        <v>1614</v>
+        <v>1643</v>
       </c>
       <c r="AM1" t="s">
-        <v>1615</v>
+        <v>1644</v>
       </c>
       <c r="AN1" t="s">
         <v>1415</v>
@@ -19263,21 +19690,21 @@
         <v>1511</v>
       </c>
       <c r="AP1" t="s">
-        <v>1565</v>
+        <v>1589</v>
       </c>
       <c r="AQ1" t="s">
-        <v>1566</v>
+        <v>1590</v>
       </c>
       <c r="AR1" t="s">
-        <v>1567</v>
+        <v>1591</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1591</v>
+        <v>1620</v>
       </c>
       <c r="B2" t="s">
-        <v>1585</v>
+        <v>1614</v>
       </c>
       <c r="C2" t="s">
         <v>1363</v>
@@ -19313,7 +19740,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="s">
-        <v>1607</v>
+        <v>1636</v>
       </c>
       <c r="O2" t="n">
         <v>12.91</v>
@@ -19408,7 +19835,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1592</v>
+        <v>1621</v>
       </c>
       <c r="B3" t="s">
         <v>1327</v>
@@ -19542,10 +19969,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1593</v>
+        <v>1622</v>
       </c>
       <c r="B4" t="s">
-        <v>1584</v>
+        <v>1613</v>
       </c>
       <c r="C4" t="s">
         <v>1365</v>
@@ -19676,10 +20103,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1594</v>
+        <v>1623</v>
       </c>
       <c r="B5" t="s">
-        <v>1585</v>
+        <v>1614</v>
       </c>
       <c r="C5" t="s">
         <v>1366</v>
@@ -19715,7 +20142,7 @@
         <v>0</v>
       </c>
       <c r="N5" t="s">
-        <v>1607</v>
+        <v>1636</v>
       </c>
       <c r="O5" t="n">
         <v>8.545</v>
@@ -19810,10 +20237,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1595</v>
+        <v>1624</v>
       </c>
       <c r="B6" t="s">
-        <v>1585</v>
+        <v>1614</v>
       </c>
       <c r="C6" t="s">
         <v>1367</v>
@@ -19849,7 +20276,7 @@
         <v>0</v>
       </c>
       <c r="N6" t="s">
-        <v>1607</v>
+        <v>1636</v>
       </c>
       <c r="O6" t="n">
         <v>7.805</v>
@@ -19944,10 +20371,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>1596</v>
+        <v>1625</v>
       </c>
       <c r="B7" t="s">
-        <v>1585</v>
+        <v>1614</v>
       </c>
       <c r="C7" t="s">
         <v>1368</v>
@@ -19983,7 +20410,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="s">
-        <v>1607</v>
+        <v>1636</v>
       </c>
       <c r="O7" t="n">
         <v>10.162</v>
@@ -20078,10 +20505,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>1597</v>
+        <v>1626</v>
       </c>
       <c r="B8" t="s">
-        <v>1585</v>
+        <v>1614</v>
       </c>
       <c r="C8" t="s">
         <v>1369</v>
@@ -20117,7 +20544,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="s">
-        <v>1607</v>
+        <v>1636</v>
       </c>
       <c r="O8" t="n">
         <v>8.538</v>
@@ -20212,10 +20639,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>1598</v>
+        <v>1627</v>
       </c>
       <c r="B9" t="s">
-        <v>1584</v>
+        <v>1613</v>
       </c>
       <c r="C9" t="s">
         <v>1370</v>
@@ -20346,10 +20773,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>1599</v>
+        <v>1628</v>
       </c>
       <c r="B10" t="s">
-        <v>1585</v>
+        <v>1614</v>
       </c>
       <c r="C10" t="s">
         <v>1371</v>
@@ -20385,7 +20812,7 @@
         <v>0</v>
       </c>
       <c r="N10" t="s">
-        <v>1607</v>
+        <v>1636</v>
       </c>
       <c r="O10" t="n">
         <v>10.575</v>
@@ -20480,7 +20907,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>1600</v>
+        <v>1629</v>
       </c>
       <c r="B11" t="s">
         <v>1327</v>
@@ -20617,7 +21044,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:H2"/>
   <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
@@ -20640,10 +21067,10 @@
         <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>1617</v>
+        <v>1646</v>
       </c>
       <c r="D1" t="s">
-        <v>1618</v>
+        <v>1647</v>
       </c>
       <c r="E1" t="s">
         <v>6</v>
@@ -20652,15 +21079,15 @@
         <v>1414</v>
       </c>
       <c r="G1" t="s">
-        <v>1620</v>
+        <v>1649</v>
       </c>
       <c r="H1" t="s">
-        <v>1621</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1616</v>
+        <v>1645</v>
       </c>
       <c r="B2" t="s">
         <v>1324</v>
@@ -20672,7 +21099,7 @@
         <v>794</v>
       </c>
       <c r="E2" t="s">
-        <v>1619</v>
+        <v>1648</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -20689,7 +21116,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:H9"/>
   <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
@@ -20712,7 +21139,7 @@
         <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>1630</v>
+        <v>1659</v>
       </c>
       <c r="D1" t="s">
         <v>6</v>
@@ -20721,18 +21148,18 @@
         <v>1414</v>
       </c>
       <c r="F1" t="s">
-        <v>1631</v>
+        <v>1660</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>201</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>1632</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1622</v>
+        <v>1651</v>
       </c>
       <c r="B2" t="s">
         <v>1324</v>
@@ -20750,15 +21177,15 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>1616</v>
+        <v>1645</v>
       </c>
       <c r="H2" t="s">
-        <v>1633</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1623</v>
+        <v>1652</v>
       </c>
       <c r="B3" t="s">
         <v>1324</v>
@@ -20776,15 +21203,15 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>1616</v>
+        <v>1645</v>
       </c>
       <c r="H3" t="s">
-        <v>1634</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1624</v>
+        <v>1653</v>
       </c>
       <c r="B4" t="s">
         <v>1324</v>
@@ -20802,15 +21229,15 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>1616</v>
+        <v>1645</v>
       </c>
       <c r="H4" t="s">
-        <v>1635</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1625</v>
+        <v>1654</v>
       </c>
       <c r="B5" t="s">
         <v>1324</v>
@@ -20828,15 +21255,15 @@
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>1616</v>
+        <v>1645</v>
       </c>
       <c r="H5" t="s">
-        <v>1636</v>
+        <v>1665</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1626</v>
+        <v>1655</v>
       </c>
       <c r="B6" t="s">
         <v>1324</v>
@@ -20854,15 +21281,15 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>1616</v>
+        <v>1645</v>
       </c>
       <c r="H6" t="s">
-        <v>1637</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>1627</v>
+        <v>1656</v>
       </c>
       <c r="B7" t="s">
         <v>1324</v>
@@ -20880,15 +21307,15 @@
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>1616</v>
+        <v>1645</v>
       </c>
       <c r="H7" t="s">
-        <v>1638</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>1628</v>
+        <v>1657</v>
       </c>
       <c r="B8" t="s">
         <v>1324</v>
@@ -20906,15 +21333,15 @@
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>1616</v>
+        <v>1645</v>
       </c>
       <c r="H8" t="s">
-        <v>1639</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>1629</v>
+        <v>1658</v>
       </c>
       <c r="B9" t="s">
         <v>1324</v>
@@ -20932,10 +21359,10 @@
         <v>0</v>
       </c>
       <c r="G9" t="s">
-        <v>1616</v>
+        <v>1645</v>
       </c>
       <c r="H9" t="s">
-        <v>1640</v>
+        <v>1669</v>
       </c>
     </row>
   </sheetData>
@@ -20943,148 +21370,175 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" bestFit="true" width="22.2421875" hidden="false" outlineLevel="0"/>
-    <col min="2" max="2" bestFit="true" width="8.76171875" hidden="false" outlineLevel="0"/>
+    <col min="1" max="1" bestFit="true" width="9.390625" hidden="false" outlineLevel="0"/>
+    <col min="2" max="2" bestFit="true" width="4.7109375" hidden="false" outlineLevel="0"/>
+    <col min="3" max="3" bestFit="true" width="22.58203125" hidden="false" outlineLevel="0"/>
+    <col min="4" max="4" bestFit="true" width="20.9140625" hidden="false" outlineLevel="0"/>
+    <col min="5" max="5" bestFit="true" width="4.03125" hidden="false" outlineLevel="0"/>
+    <col min="6" max="6" bestFit="true" width="14.68359375" hidden="false" outlineLevel="0"/>
+    <col min="7" max="7" bestFit="true" width="19.50390625" hidden="false" outlineLevel="0"/>
+    <col min="8" max="8" bestFit="true" width="17.83203125" hidden="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
-        <v>221</v>
+      <c r="A1" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>1326</v>
+        <v>11</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1675</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1676</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1414</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1677</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1678</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1641</v>
+        <v>1670</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1324</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1642</v>
+        <v>1671</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1324</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>221</v>
+        <v>1672</v>
       </c>
       <c r="B4" t="s">
-        <v>1327</v>
+        <v>1324</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="n">
+        <v>90</v>
+      </c>
+      <c r="E4" t="s">
+        <v>1324</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H4" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1639</v>
+        <v>1673</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="n">
+        <v>90</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1324</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1640</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>221</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1328</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>1637</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>1634</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>1635</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>1636</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>1633</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>1638</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>221</v>
-      </c>
-      <c r="B14" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>1643</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s">
-        <v>1644</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>1645</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>221</v>
-      </c>
-      <c r="B18" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s">
-        <v>1646</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s">
-        <v>1648</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>1649</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>1650</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="s">
-        <v>1651</v>
+        <v>1674</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" t="n">
+        <v>90</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1324</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="n">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -23672,6 +24126,350 @@
       </c>
       <c r="C271" t="s">
         <v>1318</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" width="7.28125" hidden="false" outlineLevel="0"/>
+    <col min="2" max="2" bestFit="true" width="4.7109375" hidden="false" outlineLevel="0"/>
+    <col min="3" max="3" bestFit="true" width="13.58203125" hidden="false" outlineLevel="0"/>
+    <col min="4" max="4" bestFit="true" width="4.03125" hidden="false" outlineLevel="0"/>
+    <col min="5" max="5" bestFit="true" width="15.171875" hidden="false" outlineLevel="0"/>
+    <col min="6" max="6" bestFit="true" width="19.1640625" hidden="false" outlineLevel="0"/>
+    <col min="7" max="7" bestFit="true" width="5.65234375" hidden="false" outlineLevel="0"/>
+    <col min="8" max="8" bestFit="true" width="11.5625" hidden="false" outlineLevel="0"/>
+    <col min="9" max="9" bestFit="true" width="11.57421875" hidden="false" outlineLevel="0"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1684</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1685</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1686</v>
+      </c>
+      <c r="G1" t="s">
+        <v>195</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>1679</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1324</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1687</v>
+      </c>
+      <c r="G2" t="s">
+        <v>794</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1670</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>1680</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1324</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1688</v>
+      </c>
+      <c r="G3" t="s">
+        <v>794</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1671</v>
+      </c>
+      <c r="I3" t="s">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>1681</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1324</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1689</v>
+      </c>
+      <c r="G4" t="s">
+        <v>808</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1672</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>1682</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1324</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1689</v>
+      </c>
+      <c r="G5" t="s">
+        <v>808</v>
+      </c>
+      <c r="H5" t="s">
+        <v>1673</v>
+      </c>
+      <c r="I5" t="s">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>1683</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1324</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1689</v>
+      </c>
+      <c r="G6" t="s">
+        <v>808</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1674</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1690</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" width="22.2421875" hidden="false" outlineLevel="0"/>
+    <col min="2" max="2" bestFit="true" width="8.76171875" hidden="false" outlineLevel="0"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1326</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>1691</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1327</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>1668</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>1669</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>221</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1328</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>1666</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>1663</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>1664</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>1665</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>1662</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>1667</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>221</v>
+      </c>
+      <c r="B14" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>1693</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>1695</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>221</v>
+      </c>
+      <c r="B18" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>1696</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>1697</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>1698</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>1701</v>
       </c>
     </row>
   </sheetData>

</xml_diff>